<commit_message>
Third commit – Lichee rv dock i2c configured and tested oled screen (ssd1306).
</commit_message>
<xml_diff>
--- a/Docs/Requirements.xlsx
+++ b/Docs/Requirements.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="92">
   <si>
     <t xml:space="preserve">Module</t>
   </si>
@@ -60,6 +60,9 @@
   </si>
   <si>
     <t xml:space="preserve">Developer – Dev phase 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ok</t>
   </si>
   <si>
     <t xml:space="preserve">ESP32 UART Out</t>
@@ -752,7 +755,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:H1002"/>
+  <dimension ref="B2:I1002"/>
   <sheetFormatPr defaultColWidth="14.4296875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.7"/>
@@ -808,214 +811,223 @@
         <v>12</v>
       </c>
       <c r="H3" s="6"/>
+      <c r="I3" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H4" s="9"/>
+      <c r="I4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="C4" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5" s="8" t="s">
         <v>12</v>
       </c>
       <c r="H5" s="9"/>
+      <c r="I5" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G6" s="8" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D7" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="H7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" s="8" t="s">
         <v>35</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D8" s="8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>34</v>
       </c>
       <c r="H8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D9" s="8" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E9" s="8" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D10" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G10" s="8" t="s">
         <v>46</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="E10" s="8" t="s">
-        <v>49</v>
-      </c>
-      <c r="F10" s="8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>45</v>
       </c>
       <c r="H10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G11" s="8" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="H12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H13" s="12"/>
     </row>
@@ -2024,118 +2036,118 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="13"/>
       <c r="C3" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="13"/>
       <c r="C4" s="15" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="13"/>
       <c r="C6" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="13"/>
       <c r="C8" s="14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13"/>
       <c r="C9" s="14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="13"/>
       <c r="C10" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="13"/>
       <c r="C12" s="14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D12" s="17"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="13"/>
       <c r="C13" s="15" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="13" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="13"/>
       <c r="C15" s="15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="13"/>
       <c r="C16" s="18" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="13" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="13"/>
       <c r="C18" s="19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Fourth commit – Lichee rv dock UART configured, tested data send and receive with ESP32. Data parsed and showed with oled screen (ssd1306).
</commit_message>
<xml_diff>
--- a/Docs/Requirements.xlsx
+++ b/Docs/Requirements.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="92">
   <si>
     <t xml:space="preserve">Module</t>
   </si>
@@ -815,7 +815,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
@@ -883,6 +883,9 @@
         <v>19</v>
       </c>
       <c r="H6" s="9"/>
+      <c r="I6" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="3" t="s">
@@ -904,6 +907,9 @@
         <v>35</v>
       </c>
       <c r="H7" s="9"/>
+      <c r="I7" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
@@ -925,6 +931,9 @@
         <v>35</v>
       </c>
       <c r="H8" s="9"/>
+      <c r="I8" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="3" t="s">

</xml_diff>

<commit_message>
Fifth commit – Lichee rv dock server tested, A script was implemented that loads an http server from the lichee rv dock on port 1234, displays temperature and humidity data from the data.txt file and updates it every 5 seconds. Also the main README.md file was updated.
</commit_message>
<xml_diff>
--- a/Docs/Requirements.xlsx
+++ b/Docs/Requirements.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="93">
   <si>
     <t xml:space="preserve">Module</t>
   </si>
@@ -162,6 +162,9 @@
   </si>
   <si>
     <t xml:space="preserve">Developer – Dev phase 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">x</t>
   </si>
   <si>
     <t xml:space="preserve">HTTP Server Script Test</t>
@@ -955,43 +958,49 @@
         <v>46</v>
       </c>
       <c r="H9" s="9"/>
+      <c r="I9" s="1" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10" s="8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" s="8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G10" s="8" t="s">
         <v>46</v>
       </c>
       <c r="H10" s="9"/>
+      <c r="I10" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D11" s="8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E11" s="8" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>46</v>
@@ -1000,43 +1009,46 @@
     </row>
     <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E12" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F12" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G12" s="8" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H12" s="9"/>
+      <c r="I12" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H13" s="12"/>
     </row>
@@ -2045,118 +2057,118 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="13"/>
       <c r="C3" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="13"/>
       <c r="C4" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="13"/>
       <c r="C6" s="14" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="13"/>
       <c r="C8" s="14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13"/>
       <c r="C9" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="13"/>
       <c r="C10" s="14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="13"/>
       <c r="C12" s="14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="D12" s="17"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="13"/>
       <c r="C13" s="15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="13" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="13"/>
       <c r="C15" s="15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="13"/>
       <c r="C16" s="18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="13" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="13"/>
       <c r="C18" s="19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Six commit – Lichee rv dock server as service implemented, also was implemented a led pilot as service to verify system unbug. Main README.md updated and wiring diagram upload. this project version includes all features and works auto mode
</commit_message>
<xml_diff>
--- a/Docs/Requirements.xlsx
+++ b/Docs/Requirements.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="93">
   <si>
     <t xml:space="preserve">Module</t>
   </si>
@@ -1006,6 +1006,9 @@
         <v>46</v>
       </c>
       <c r="H11" s="9"/>
+      <c r="I11" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
@@ -1051,6 +1054,9 @@
         <v>69</v>
       </c>
       <c r="H13" s="12"/>
+      <c r="I13" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>

<commit_message>
Last commit, The requirement check list was verified by Leandro Zapata, classmate
</commit_message>
<xml_diff>
--- a/Docs/Requirements.xlsx
+++ b/Docs/Requirements.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="90">
   <si>
     <t xml:space="preserve">Module</t>
   </si>
@@ -38,10 +38,10 @@
     <t xml:space="preserve">Success Criteria</t>
   </si>
   <si>
-    <t xml:space="preserve">Run (Who/When)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Checked ✔️</t>
+    <t xml:space="preserve">Run (Who)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Checked by Leandro Zapata / 18 de Julio 2025</t>
   </si>
   <si>
     <t xml:space="preserve">ESP32 I2C Init</t>
@@ -59,7 +59,10 @@
     <t xml:space="preserve"> Data obtain on terminal logs</t>
   </si>
   <si>
-    <t xml:space="preserve">Developer – Dev phase 1</t>
+    <t xml:space="preserve">Yonnier Muñoz</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✔️</t>
   </si>
   <si>
     <t xml:space="preserve">ok</t>
@@ -80,9 +83,6 @@
     <t xml:space="preserve">Data in format XX.X,YY.Y </t>
   </si>
   <si>
-    <t xml:space="preserve">Developer – Dev phase 2</t>
-  </si>
-  <si>
     <t xml:space="preserve">Lichee I2C Init</t>
   </si>
   <si>
@@ -128,9 +128,6 @@
     <t xml:space="preserve">Parsed values match what ESP32 sends</t>
   </si>
   <si>
-    <t xml:space="preserve">Developer – Dev phase 3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Display Update</t>
   </si>
   <si>
@@ -161,7 +158,7 @@
     <t xml:space="preserve">Another device can connect to SSID and ping ip</t>
   </si>
   <si>
-    <t xml:space="preserve">Developer – Dev phase 4</t>
+    <t xml:space="preserve">It was not implemented because the web server can be operated using the lichee in station mode.</t>
   </si>
   <si>
     <t xml:space="preserve">x</t>
@@ -212,9 +209,6 @@
     <t xml:space="preserve">Display updates without manual run</t>
   </si>
   <si>
-    <t xml:space="preserve">Developer – Final integration</t>
-  </si>
-  <si>
     <t xml:space="preserve">Full Integration</t>
   </si>
   <si>
@@ -228,9 +222,6 @@
   </si>
   <si>
     <t xml:space="preserve">Sensor values displayed locally + on web</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dev + Test Team – Final milestone</t>
   </si>
   <si>
     <t xml:space="preserve">Hardware Setup</t>
@@ -309,7 +300,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +330,13 @@
       <name val="Calibri"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -513,7 +511,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -525,7 +523,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -537,7 +535,7 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -768,10 +766,11 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="26.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="20.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="19.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="8" style="1" width="10.7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="21.32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="9" style="1" width="10.7"/>
   </cols>
   <sheetData>
-    <row r="2" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -813,33 +812,37 @@
       <c r="G3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H3" s="6"/>
+      <c r="H3" s="6" t="s">
+        <v>13</v>
+      </c>
       <c r="I3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="1" t="s">
         <v>14</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H4" s="9"/>
-      <c r="I4" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -858,12 +861,14 @@
       <c r="F5" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="G5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="9"/>
+      <c r="H5" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="I5" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -882,12 +887,14 @@
       <c r="F6" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="G6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H6" s="9"/>
+      <c r="G6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="I6" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -906,156 +913,168 @@
       <c r="F7" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G7" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="H7" s="9"/>
+      <c r="G7" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="I7" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="D8" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="E8" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="8" t="s">
+      <c r="F8" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="F8" s="8" t="s">
+      <c r="G8" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="47.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B9" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="G8" s="8" t="s">
-        <v>35</v>
-      </c>
-      <c r="H8" s="9"/>
-      <c r="I8" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="E9" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="8" t="s">
+      <c r="F9" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="G9" s="8" t="s">
+      <c r="H9" s="5"/>
+      <c r="I9" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="H9" s="9"/>
-      <c r="I9" s="1" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="D10" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="E10" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="F10" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="F10" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="G10" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H10" s="9"/>
+      <c r="G10" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="I10" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="7" t="s">
+      <c r="D11" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="8" t="s">
+      <c r="E11" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="8" t="s">
+      <c r="F11" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="F11" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="G11" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H11" s="9"/>
+      <c r="G11" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="I11" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="D12" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="8" t="s">
+      <c r="E12" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="F12" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="F12" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="G12" s="8" t="s">
-        <v>63</v>
-      </c>
-      <c r="H12" s="9"/>
+      <c r="G12" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="I12" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="E13" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="F13" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>67</v>
-      </c>
-      <c r="F13" s="11" t="s">
-        <v>68</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="H13" s="12"/>
+      <c r="G13" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>13</v>
+      </c>
       <c r="I13" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2039,6 +2058,9 @@
     <row r="1001" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1002" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="G9:H9"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2063,118 +2085,118 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="13" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C2" s="14" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="13"/>
       <c r="C3" s="14" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="13"/>
       <c r="C4" s="15" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="13" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="13"/>
       <c r="C6" s="14" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="13" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="13"/>
       <c r="C8" s="14" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="13"/>
       <c r="C9" s="14" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="13"/>
       <c r="C10" s="14" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="13"/>
       <c r="C12" s="14" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D12" s="17"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="13"/>
       <c r="C13" s="15" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="13" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="D14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="13"/>
       <c r="C15" s="15" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="13"/>
       <c r="C16" s="18" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="13" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C17" s="16" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="13"/>
       <c r="C18" s="19" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>